<commit_message>
adding eleonora top choices for GPT queries
</commit_message>
<xml_diff>
--- a/experiment/instructions/ai_query_11_classified.xlsx
+++ b/experiment/instructions/ai_query_11_classified.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elfre4573/Documents/GitHub/AI_advice/experiment/instructions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BDF674-1AB9-1243-88B0-9D62C319BCB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB1DAD38-CF68-9147-A0D8-696B8DB9DD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="give 3" sheetId="2" r:id="rId1"/>
     <sheet name="give 3 - full sentence" sheetId="7" r:id="rId2"/>
-    <sheet name="give 0" sheetId="6" r:id="rId3"/>
-    <sheet name="take 4" sheetId="4" r:id="rId4"/>
-    <sheet name="others" sheetId="3" r:id="rId5"/>
+    <sheet name="Eleonora top choices" sheetId="8" r:id="rId3"/>
+    <sheet name="give 0" sheetId="6" r:id="rId4"/>
+    <sheet name="take 4" sheetId="4" r:id="rId5"/>
+    <sheet name="others" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'give 0'!$A$1:$D$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'give 0'!$A$1:$D$159</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'give 3 - full sentence'!$A$1:$D$96</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="795">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="795">
   <si>
     <t>Evaluative Standard: Ethical Egalitarianism, aiming for equal distribution
 Recommendation: The decision-maker should give $3 to the recipient. 
@@ -5578,6 +5579,162 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2AC988-BEEA-9244-BA2F-7C0ABFE03798}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.5" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.5" customWidth="1"/>
+    <col min="4" max="4" width="31.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="154" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
+        <v>672</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>679</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="126" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>672</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>680</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="154" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>713</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="140" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>783</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>781</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>784</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="154" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
+        <v>717</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>719</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="126" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>717</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>722</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="154" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>723</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>724</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="140" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
+        <v>723</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>725</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="140" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>727</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>729</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0700F54-0547-5A4F-A343-D6F4173ABBD3}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:D159"/>
@@ -7810,7 +7967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{399103A6-82F6-5B41-8361-39C43BF895A7}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -7838,7 +7995,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F224ACC2-145B-384E-88BE-AC5A7C03AD84}">
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>